<commit_message>
CAPPED version + other stuff
</commit_message>
<xml_diff>
--- a/results/results_diabetes_korea_simple.xlsx
+++ b/results/results_diabetes_korea_simple.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AO3"/>
+  <dimension ref="A1:AR3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -422,140 +422,155 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
+          <t>med_cap</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>D_years</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>deaths</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>seyll</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>YLD_sex</t>
-        </is>
-      </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
+          <t>YLD_mode</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>YLD_lower</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>YLD_upper</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
           <t>PAF_med</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>PAF_lo</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>PAF_hi</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>AC_med</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>AC_lo</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>AC_hi</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>AD_med</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>AD_lo</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>AD_hi</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>YLD_incidence_med</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>YLD_incidence_lo</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>YLD_incidence_hi</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>YLD_prevalence_med</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>YLD_prevalence_lo</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>YLD_prevalence_hi</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>YLL_med</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>YLL_lo</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>YLL_hi</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>DALY_incidence_med</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>DALY_incidence_lo</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>DALY_incidence_hi</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>DALY_prevalence_med</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>DALY_prevalence_lo</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>DALY_prevalence_hi</t>
         </is>
@@ -604,88 +619,97 @@
         <v>0.18</v>
       </c>
       <c r="N2">
+        <v>0.1732661337461954</v>
+      </c>
+      <c r="O2">
         <v>19.10000000000001</v>
       </c>
-      <c r="O2">
+      <c r="P2">
         <v>599.79</v>
       </c>
-      <c r="P2">
+      <c r="Q2">
         <v>13.16585805031761</v>
       </c>
-      <c r="Q2">
+      <c r="R2">
         <v>8355.608426829789</v>
       </c>
-      <c r="R2">
-        <v>0.5655118872499525</v>
-      </c>
       <c r="S2">
-        <v>0.1748659382502645</v>
+        <v>5617.300593266269</v>
       </c>
       <c r="T2">
-        <v>0.7759762354111954</v>
+        <v>11465.14910195645</v>
       </c>
       <c r="U2">
-        <v>2860.359125710259</v>
+        <v>0.5468342732675411</v>
       </c>
       <c r="V2">
-        <v>884.4719156698376</v>
+        <v>0.1230068841019617</v>
       </c>
       <c r="W2">
-        <v>3924.887798709826</v>
+        <v>0.7571894554780508</v>
       </c>
       <c r="X2">
-        <v>339.188374853649</v>
+        <v>2765.887754187223</v>
       </c>
       <c r="Y2">
-        <v>104.8828411031261</v>
+        <v>622.1688197877224</v>
       </c>
       <c r="Z2">
-        <v>465.4227862372808</v>
+        <v>3829.864265807981</v>
       </c>
       <c r="AA2">
-        <v>3640.762118546997</v>
+        <v>327.9857287631385</v>
       </c>
       <c r="AB2">
-        <v>1070.675803783273</v>
+        <v>73.77829901551563</v>
       </c>
       <c r="AC2">
-        <v>6032.755508858303</v>
+        <v>454.15466350118</v>
       </c>
       <c r="AD2">
-        <v>4725.19589057812</v>
+        <v>3534.187397499984</v>
       </c>
       <c r="AE2">
-        <v>1461.111307209407</v>
+        <v>761.8226371799839</v>
       </c>
       <c r="AF2">
-        <v>6483.753571621441</v>
+        <v>5939.730529890795</v>
       </c>
       <c r="AG2">
-        <v>4465.705995641061</v>
+        <v>4463.571812799732</v>
       </c>
       <c r="AH2">
-        <v>1380.872597877776</v>
+        <v>1003.932538464221</v>
       </c>
       <c r="AI2">
-        <v>6127.690336983356</v>
+        <v>6867.83710839018</v>
       </c>
       <c r="AJ2">
-        <v>8204.592613404653</v>
+        <v>4318.213547425456</v>
       </c>
       <c r="AK2">
-        <v>2533.328470955399</v>
+        <v>971.3546120321663</v>
       </c>
       <c r="AL2">
-        <v>11979.48258204531</v>
+        <v>5979.335832546297</v>
       </c>
       <c r="AM2">
-        <v>9190.901886219181</v>
+        <v>7886.036904286856</v>
       </c>
       <c r="AN2">
-        <v>2841.983905087183</v>
+        <v>1708.77613265136</v>
       </c>
       <c r="AO2">
-        <v>12611.4439086048</v>
+        <v>11727.27152943065</v>
+      </c>
+      <c r="AP2">
+        <v>8802.430707795733</v>
+      </c>
+      <c r="AQ2">
+        <v>1944.400772079556</v>
+      </c>
+      <c r="AR2">
+        <v>12601.50711886464</v>
       </c>
     </row>
     <row r="3">
@@ -731,88 +755,97 @@
         <v>0.29</v>
       </c>
       <c r="N3">
+        <v>0.1732661337461954</v>
+      </c>
+      <c r="O3">
         <v>17.8</v>
       </c>
-      <c r="O3">
+      <c r="P3">
         <v>783.0599999999999</v>
       </c>
-      <c r="P3">
+      <c r="Q3">
         <v>16.50964166219702</v>
       </c>
-      <c r="Q3">
+      <c r="R3">
         <v>13225.90447579696</v>
       </c>
-      <c r="R3">
-        <v>0.7740105214427841</v>
-      </c>
       <c r="S3">
-        <v>0.1875409158649912</v>
+        <v>8916.644865520693</v>
       </c>
       <c r="T3">
-        <v>0.9254013542795342</v>
+        <v>17957.83716914366</v>
       </c>
       <c r="U3">
-        <v>6257.101055343466</v>
+        <v>0.5570496113494856</v>
       </c>
       <c r="V3">
-        <v>1516.080763852588</v>
+        <v>0.187649500168478</v>
       </c>
       <c r="W3">
-        <v>7480.944547995755</v>
+        <v>0.7777807203980891</v>
       </c>
       <c r="X3">
-        <v>606.0966789209865</v>
+        <v>4503.189058149241</v>
       </c>
       <c r="Y3">
-        <v>146.85578957724</v>
+        <v>1516.958559361976</v>
       </c>
       <c r="Z3">
-        <v>724.644784482132</v>
+        <v>6287.579343698152</v>
       </c>
       <c r="AA3">
-        <v>7251.602020337377</v>
+        <v>436.2032686633281</v>
       </c>
       <c r="AB3">
-        <v>1952.634662941015</v>
+        <v>146.9408176019284</v>
       </c>
       <c r="AC3">
-        <v>11345.60598622314</v>
+        <v>609.0489709149276</v>
       </c>
       <c r="AD3">
-        <v>10236.98921986406</v>
+        <v>5354.774938319879</v>
       </c>
       <c r="AE3">
-        <v>2480.398238533848</v>
+        <v>1767.869300135417</v>
       </c>
       <c r="AF3">
-        <v>12239.26991347426</v>
+        <v>8857.201371976022</v>
       </c>
       <c r="AG3">
-        <v>10006.43898163317</v>
+        <v>7200.212603762933</v>
       </c>
       <c r="AH3">
-        <v>2424.53646193924</v>
+        <v>2289.962316690566</v>
       </c>
       <c r="AI3">
-        <v>11963.62572417999</v>
+        <v>11366.62840959124</v>
       </c>
       <c r="AJ3">
-        <v>17313.6241591019</v>
+        <v>7201.559657510604</v>
       </c>
       <c r="AK3">
-        <v>4279.892376844336</v>
+        <v>2425.94024415809</v>
       </c>
       <c r="AL3">
-        <v>22628.46370817224</v>
+        <v>10055.18026453531</v>
       </c>
       <c r="AM3">
-        <v>20243.42820149723</v>
+        <v>12667.3265505709</v>
       </c>
       <c r="AN3">
-        <v>4904.934700473089</v>
+        <v>4266.350013160704</v>
       </c>
       <c r="AO3">
-        <v>24202.89563765425</v>
+        <v>18169.03426244861</v>
+      </c>
+      <c r="AP3">
+        <v>14488.1320491846</v>
+      </c>
+      <c r="AQ3">
+        <v>4822.265981414587</v>
+      </c>
+      <c r="AR3">
+        <v>21063.46575576582</v>
       </c>
     </row>
   </sheetData>

</xml_diff>